<commit_message>
prolif started IFPs logistic regression model, ligand names in .pkls
</commit_message>
<xml_diff>
--- a/AUC_stats.xlsx
+++ b/AUC_stats.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BABCA4C0-9522-4044-A787-97BFF84B9BD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="18020" yWindow="800" windowWidth="17620" windowHeight="21380" xr2:uid="{7AE26DC2-4DB2-7340-96F1-86A28CD7C8BC}"/>
+    <workbookView xWindow="23920" yWindow="800" windowWidth="11720" windowHeight="21380" xr2:uid="{7AE26DC2-4DB2-7340-96F1-86A28CD7C8BC}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1890,6 +1890,18 @@
       <c r="K65" s="2"/>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="B4:K6 B8:K10">
+    <cfRule type="colorScale" priority="4">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="num" val="80"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="B4:K6 L5:L7 B8:K10">
     <cfRule type="colorScale" priority="9">
       <colorScale>
@@ -1902,8 +1914,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B4:K6 B8:K10">
-    <cfRule type="colorScale" priority="4">
+  <conditionalFormatting sqref="B7:K7">
+    <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="percentile" val="50"/>
@@ -1916,6 +1928,18 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="B15:K17 B19:K21">
     <cfRule type="colorScale" priority="8">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF5A8AC6"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B18:K18">
+    <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -1950,30 +1974,6 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B7:K7">
-    <cfRule type="colorScale" priority="2">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="num" val="80"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B18:K18">
-    <cfRule type="colorScale" priority="1">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF5A8AC6"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="H3" r:id="rId1" display="6TVE_C_@" xr:uid="{77561480-A1A3-0142-8D0A-C9E5CCFA5804}"/>
     <hyperlink ref="H14" r:id="rId2" display="6TVE_C_@" xr:uid="{0A740804-6500-4941-B93E-98E80738321B}"/>

</xml_diff>